<commit_message>
build: MGF 리포트 2026-06-10 최신화
</commit_message>
<xml_diff>
--- a/reports/셀린느/셀린느_league_mgf_report.xlsx
+++ b/reports/셀린느/셀린느_league_mgf_report.xlsx
@@ -10,15 +10,15 @@
     <sheet name="guilds" sheetId="1" r:id="rId1"/>
     <sheet name="셀린느" sheetId="2" r:id="rId2"/>
     <sheet name="호러" sheetId="3" r:id="rId3"/>
-    <sheet name="딸기키우기" sheetId="4" r:id="rId4"/>
-    <sheet name="LUXURY" sheetId="5" r:id="rId5"/>
+    <sheet name="LUXURY" sheetId="4" r:id="rId4"/>
+    <sheet name="딸기키우기" sheetId="5" r:id="rId5"/>
     <sheet name="item" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">guilds!$A$1:$M$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">item!$A$1:$J$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">LUXURY!$A$1:$J$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">딸기키우기!$A$1:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">LUXURY!$A$1:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">딸기키우기!$A$1:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">셀린느!$A$1:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">호러!$A$1:$J$31</definedName>
   </definedNames>
@@ -80,495 +80,498 @@
     <t>Scania 2</t>
   </si>
   <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>1위</t>
+  </si>
+  <si>
+    <t>Lv.9</t>
+  </si>
+  <si>
+    <t>30명</t>
+  </si>
+  <si>
+    <t>19경 2080조 4912억 2112만</t>
+  </si>
+  <si>
+    <t>[통합2섭1위] [토벌전1위 최종뎀10%][IN50위] 문의 [혜영]</t>
+  </si>
+  <si>
+    <t>혜영</t>
+  </si>
+  <si>
+    <t>2026.06.10</t>
+  </si>
+  <si>
+    <t>호러</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/guild_info.php?g_name=%ED%98%B8%EB%9F%AC</t>
+  </si>
+  <si>
+    <t>Scania 10</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>Lv.8</t>
+  </si>
+  <si>
+    <t>22경 5150조 601억 2172만</t>
+  </si>
+  <si>
+    <t>오래 하실분들 환영입니다</t>
+  </si>
+  <si>
+    <t>기요밋</t>
+  </si>
+  <si>
+    <t>LUXURY</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/guild_info.php?g_name=LUXURY</t>
+  </si>
+  <si>
+    <t>Scania 16</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>12경 4301조 343억 8536만</t>
+  </si>
+  <si>
+    <t>*[100LV] 이상/활동,일일 업그레이드 필수* 대기 가능 문의 귓</t>
+  </si>
+  <si>
+    <t>살뽀시</t>
+  </si>
+  <si>
+    <t>딸기키우기</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/guild_info.php?g_name=%EB%94%B8%EA%B8%B0%ED%82%A4%EC%9A%B0%EA%B8%B0</t>
+  </si>
+  <si>
+    <t>Scania 28</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>3위</t>
+  </si>
+  <si>
+    <t>16경 5903조 2011억 8275만</t>
+  </si>
+  <si>
+    <t>길컨에 진심인 길드입니다 300조 이상 무치z / 연지임당 으로 문의주세요</t>
+  </si>
+  <si>
+    <t>무치z</t>
+  </si>
+  <si>
+    <t>item</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/guild_info.php?g_name=item</t>
+  </si>
+  <si>
+    <t>Scania 34</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>16경 7350조 9775억 7658만</t>
+  </si>
+  <si>
+    <t>We Go Together !</t>
+  </si>
+  <si>
+    <t>토마스셸비</t>
+  </si>
+  <si>
+    <t>member_rank_in_guild</t>
+  </si>
+  <si>
+    <t>nickname</t>
+  </si>
+  <si>
+    <t>character_key</t>
+  </si>
+  <si>
+    <t>character_url</t>
+  </si>
+  <si>
+    <t>is_master</t>
+  </si>
+  <si>
+    <t>job_name</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>combat_power</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>스타냥이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%8A%A4%ED%83%80%EB%83%A5%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>신궁</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>11경 313조 6930억 1923만</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>돈스</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8F%88%EC%8A%A4</t>
+  </si>
+  <si>
+    <t>비숍</t>
+  </si>
+  <si>
+    <t>116</t>
+  </si>
+  <si>
+    <t>1경 6994조 5547억 4273만</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>말레이히어로</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A7%90%EB%A0%88%EC%9D%B4%ED%9E%88%EC%96%B4%EB%A1%9C</t>
+  </si>
+  <si>
+    <t>히어로</t>
+  </si>
+  <si>
+    <t>115</t>
+  </si>
+  <si>
+    <t>1경 4853조 2340억 7413만</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>진자이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A7%84%EC%9E%90%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>1경 1742조 9172억 2791만</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>스타캐치</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%8A%A4%ED%83%80%EC%BA%90%EC%B9%98</t>
+  </si>
+  <si>
+    <t>섀도어</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>1경 217조 1743억 7192만</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>소소채2</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%86%8C%EC%86%8C%EC%B1%842</t>
+  </si>
+  <si>
+    <t>112</t>
+  </si>
+  <si>
+    <t>3690조 9572억 3420만</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>단풍노비</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8B%A8%ED%92%8D%EB%85%B8%EB%B9%84</t>
+  </si>
+  <si>
+    <t>3444조 4147억 1811만</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>니달리신</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8B%88%EB%8B%AC%EB%A6%AC%EC%8B%A0</t>
+  </si>
+  <si>
+    <t>2474조 2569억 7280만</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>오리부엉이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%98%A4%EB%A6%AC%EB%B6%80%EC%97%89%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
+    <t>2242조 7579억 9328만</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>약어</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%95%BD%EC%96%B4</t>
+  </si>
+  <si>
+    <t>팔라딘</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>2001조 6228억 2542만</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>여사</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%97%AC%EC%82%AC</t>
+  </si>
+  <si>
+    <t>다크나이트</t>
+  </si>
+  <si>
+    <t>1800조 8206억 6812만</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>닼나짱2</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8B%BC%EB%82%98%EC%A7%B12</t>
+  </si>
+  <si>
+    <t>1754조 5435억 6825만</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>김겨탱</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%B9%80%EA%B2%A8%ED%83%B1</t>
+  </si>
+  <si>
+    <t>1591조 676억 7650만</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>꽃을든남자</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%BD%83%EC%9D%84%EB%93%A0%EB%82%A8%EC%9E%90</t>
+  </si>
+  <si>
+    <t>1216조 436억 9979만</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>두근푸근연근</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%91%90%EA%B7%BC%ED%91%B8%EA%B7%BC%EC%97%B0%EA%B7%BC</t>
+  </si>
+  <si>
+    <t>1188조 5830억 7202만</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>잼포즈</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%9E%BC%ED%8F%AC%EC%A6%88</t>
+  </si>
+  <si>
+    <t>아크메이지(썬,콜)</t>
+  </si>
+  <si>
+    <t>1080조 1881억 3755만</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>하후돈</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%95%98%ED%9B%84%EB%8F%88</t>
+  </si>
+  <si>
+    <t>1010조 7233억 7977만</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>트라이던트</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%8A%B8%EB%9D%BC%EC%9D%B4%EB%8D%98%ED%8A%B8</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>926조 9872억 3417만</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>프리프리</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%94%84%EB%A6%AC%ED%94%84%EB%A6%AC</t>
+  </si>
+  <si>
+    <t>738조 4930억 4298만</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>할룽</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%95%A0%EB%A3%BD</t>
+  </si>
+  <si>
+    <t>517조 1198억 6694만</t>
+  </si>
+  <si>
+    <t>쾌감</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%BE%8C%EA%B0%90</t>
+  </si>
+  <si>
+    <t>491조 1417억 5802만</t>
+  </si>
+  <si>
+    <t>루넨</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A3%A8%EB%84%A8</t>
+  </si>
+  <si>
+    <t>321조 4304억 9957만</t>
+  </si>
+  <si>
     <t>23</t>
   </si>
   <si>
-    <t>1위</t>
-  </si>
-  <si>
-    <t>Lv.9</t>
-  </si>
-  <si>
-    <t>30명</t>
-  </si>
-  <si>
-    <t>18경 572조 1426억 3184만</t>
-  </si>
-  <si>
-    <t>[통합2섭1위] [토벌전1위 최종뎀10%][IN50위] 문의 [혜영]</t>
-  </si>
-  <si>
-    <t>혜영</t>
-  </si>
-  <si>
-    <t>2026.06.09</t>
-  </si>
-  <si>
-    <t>호러</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/guild_info.php?g_name=%ED%98%B8%EB%9F%AC</t>
-  </si>
-  <si>
-    <t>Scania 10</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>Lv.8</t>
-  </si>
-  <si>
-    <t>21경 9603조 5094억 818만</t>
-  </si>
-  <si>
-    <t>오래 하실분들 환영입니다</t>
-  </si>
-  <si>
-    <t>기요밋</t>
-  </si>
-  <si>
-    <t>딸기키우기</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/guild_info.php?g_name=%EB%94%B8%EA%B8%B0%ED%82%A4%EC%9A%B0%EA%B8%B0</t>
-  </si>
-  <si>
-    <t>Scania 28</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>3위</t>
-  </si>
-  <si>
-    <t>16경 4944조 1669억 3875만</t>
-  </si>
-  <si>
-    <t>길컨에 진심인 길드입니다 300조 이상 무치z / 연지임당 으로 문의주세요</t>
-  </si>
-  <si>
-    <t>무치z</t>
-  </si>
-  <si>
-    <t>LUXURY</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/guild_info.php?g_name=LUXURY</t>
-  </si>
-  <si>
-    <t>Scania 16</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>12경 3056조 7170억 4889만</t>
-  </si>
-  <si>
-    <t>*[100LV] 이상/활동,일일 업그레이드 필수* 대기 가능 문의 귓</t>
-  </si>
-  <si>
-    <t>살뽀시</t>
-  </si>
-  <si>
-    <t>item</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/guild_info.php?g_name=item</t>
-  </si>
-  <si>
-    <t>Scania 34</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>16경 6221조 7690억 4390만</t>
-  </si>
-  <si>
-    <t>We Go Together !</t>
-  </si>
-  <si>
-    <t>토마스셸비</t>
-  </si>
-  <si>
-    <t>member_rank_in_guild</t>
-  </si>
-  <si>
-    <t>nickname</t>
-  </si>
-  <si>
-    <t>character_key</t>
-  </si>
-  <si>
-    <t>character_url</t>
-  </si>
-  <si>
-    <t>is_master</t>
-  </si>
-  <si>
-    <t>job_name</t>
-  </si>
-  <si>
-    <t>level</t>
-  </si>
-  <si>
-    <t>combat_power</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>스타냥이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%8A%A4%ED%83%80%EB%83%A5%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>신궁</t>
-  </si>
-  <si>
-    <t>118</t>
-  </si>
-  <si>
-    <t>10경 145조 5404억 5302만</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>돈스</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8F%88%EC%8A%A4</t>
-  </si>
-  <si>
-    <t>비숍</t>
-  </si>
-  <si>
-    <t>116</t>
-  </si>
-  <si>
-    <t>1경 6994조 5547억 4273만</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>말레이히어로</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A7%90%EB%A0%88%EC%9D%B4%ED%9E%88%EC%96%B4%EB%A1%9C</t>
-  </si>
-  <si>
-    <t>히어로</t>
-  </si>
-  <si>
-    <t>115</t>
-  </si>
-  <si>
-    <t>1경 4853조 2340억 7413만</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>진자이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A7%84%EC%9E%90%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>1경 1742조 9172억 2791만</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>스타캐치</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%8A%A4%ED%83%80%EC%BA%90%EC%B9%98</t>
-  </si>
-  <si>
-    <t>섀도어</t>
-  </si>
-  <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>9723조 3562억 7980만</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>소소채2</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%86%8C%EC%86%8C%EC%B1%842</t>
-  </si>
-  <si>
-    <t>112</t>
-  </si>
-  <si>
-    <t>3680조 7124억 9169만</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>단풍노비</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8B%A8%ED%92%8D%EB%85%B8%EB%B9%84</t>
-  </si>
-  <si>
-    <t>2908조 6504억 3357만</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>니달리신</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8B%88%EB%8B%AC%EB%A6%AC%EC%8B%A0</t>
-  </si>
-  <si>
-    <t>111</t>
-  </si>
-  <si>
-    <t>2474조 2569억 7280만</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>오리부엉이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%98%A4%EB%A6%AC%EB%B6%80%EC%97%89%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>2210조 7183억 609만</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>약어</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%95%BD%EC%96%B4</t>
-  </si>
-  <si>
-    <t>팔라딘</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>1904조 1372억 8931만</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>여사</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%97%AC%EC%82%AC</t>
-  </si>
-  <si>
-    <t>다크나이트</t>
-  </si>
-  <si>
-    <t>1800조 8206억 6812만</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>닼나짱2</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8B%BC%EB%82%98%EC%A7%B12</t>
-  </si>
-  <si>
-    <t>1754조 5435억 6825만</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>김겨탱</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%B9%80%EA%B2%A8%ED%83%B1</t>
-  </si>
-  <si>
-    <t>1591조 676억 7650만</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>꽃을든남자</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%BD%83%EC%9D%84%EB%93%A0%EB%82%A8%EC%9E%90</t>
-  </si>
-  <si>
-    <t>1213조 9719억 643만</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>두근푸근연근</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%91%90%EA%B7%BC%ED%91%B8%EA%B7%BC%EC%97%B0%EA%B7%BC</t>
-  </si>
-  <si>
-    <t>1098조 7974억 2507만</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>잼포즈</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%9E%BC%ED%8F%AC%EC%A6%88</t>
-  </si>
-  <si>
-    <t>아크메이지(썬,콜)</t>
-  </si>
-  <si>
-    <t>1078조 162억 5979만</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>하후돈</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%95%98%ED%9B%84%EB%8F%88</t>
-  </si>
-  <si>
-    <t>1010조 7233억 7977만</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>트라이던트</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%8A%B8%EB%9D%BC%EC%9D%B4%EB%8D%98%ED%8A%B8</t>
-  </si>
-  <si>
-    <t>109</t>
-  </si>
-  <si>
-    <t>888조 4320억 1692만</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>프리프리</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%94%84%EB%A6%AC%ED%94%84%EB%A6%AC</t>
-  </si>
-  <si>
-    <t>736조 4543억 3438만</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>할룽</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%95%A0%EB%A3%BD</t>
-  </si>
-  <si>
-    <t>517조 1198억 6694만</t>
-  </si>
-  <si>
-    <t>쾌감</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%BE%8C%EA%B0%90</t>
-  </si>
-  <si>
-    <t>491조 1417억 5802만</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>루넨</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A3%A8%EB%84%A8</t>
-  </si>
-  <si>
-    <t>295조 1857억 522만</t>
-  </si>
-  <si>
     <t>김치싸대기</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%EA%B9%80%EC%B9%98%EC%8B%B8%EB%8C%80%EA%B8%B0</t>
   </si>
   <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>284조 2442억 6503만</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>POSCO</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=POSCO</t>
+  </si>
+  <si>
+    <t>277조 3468억 3844만</t>
+  </si>
+  <si>
+    <t>제로슈가</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A0%9C%EB%A1%9C%EC%8A%88%EA%B0%80</t>
+  </si>
+  <si>
+    <t>아크메이지(불,독)</t>
+  </si>
+  <si>
+    <t>217조 310억 6660만</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%98%9C%EC%98%81</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
     <t>107</t>
   </si>
   <si>
-    <t>279조 8603억 3052만</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>POSCO</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=POSCO</t>
-  </si>
-  <si>
-    <t>276조 3863억 5988만</t>
-  </si>
-  <si>
-    <t>제로슈가</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A0%9C%EB%A1%9C%EC%8A%88%EA%B0%80</t>
-  </si>
-  <si>
-    <t>아크메이지(불,독)</t>
-  </si>
-  <si>
-    <t>216조 3242억 926만</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%98%9C%EC%98%81</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>200조 4270억 4898만</t>
   </si>
   <si>
@@ -593,9 +596,6 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%8C%80%EB%B0%A9%EC%96%B4%EC%A1%B0%EC%95%84</t>
   </si>
   <si>
-    <t>108</t>
-  </si>
-  <si>
     <t>132조 1666억 731만</t>
   </si>
   <si>
@@ -611,7 +611,7 @@
     <t>105</t>
   </si>
   <si>
-    <t>100조 9017억 3226만</t>
+    <t>100조 9096억 2813만</t>
   </si>
   <si>
     <t>30</t>
@@ -623,7 +623,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%AA%BD%ED%98%B8</t>
   </si>
   <si>
-    <t>79조 2037억 7012만</t>
+    <t>81조 9558억 5905만</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%EA%B8%B0%EC%9A%94%EB%B0%8B</t>
@@ -632,7 +632,7 @@
     <t>117</t>
   </si>
   <si>
-    <t>13경 5504조 4017억 1743만</t>
+    <t>14경 536조 7005억 4862만</t>
   </si>
   <si>
     <t>난풍</t>
@@ -650,7 +650,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%88%84%EC%A7%9C</t>
   </si>
   <si>
-    <t>1경 2021조 32억 4961만</t>
+    <t>1경 2050조 6733억 6861만</t>
   </si>
   <si>
     <t>일월마녀</t>
@@ -659,7 +659,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%9D%BC%EC%9B%94%EB%A7%88%EB%85%80</t>
   </si>
   <si>
-    <t>1경 149조 8833억 3583만</t>
+    <t>1경 525조 8552억 5706만</t>
   </si>
   <si>
     <t>로드숍</t>
@@ -680,7 +680,7 @@
     <t>113</t>
   </si>
   <si>
-    <t>4542조 4624억 3551만</t>
+    <t>4543조 373억 9518만</t>
   </si>
   <si>
     <t>피몽</t>
@@ -698,7 +698,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%A7%84%EC%A7%9C%EC%A7%80%EC%A1%B4%EB%B2%95%EC%82%AC</t>
   </si>
   <si>
-    <t>1218조 1974억 5537만</t>
+    <t>1220조 70억 1080만</t>
   </si>
   <si>
     <t>다이사</t>
@@ -707,7 +707,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%8B%A4%EC%9D%B4%EC%82%AC</t>
   </si>
   <si>
-    <t>1137조 5875억 6120만</t>
+    <t>1141조 3934억 2660만</t>
   </si>
   <si>
     <t>똥으리</t>
@@ -737,6 +737,15 @@
     <t>628조 1615억 4796만</t>
   </si>
   <si>
+    <t>고래털</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%B3%A0%EB%9E%98%ED%84%B8</t>
+  </si>
+  <si>
+    <t>319조 7939억 3022만</t>
+  </si>
+  <si>
     <t>태켱</t>
   </si>
   <si>
@@ -746,22 +755,13 @@
     <t>311조 8170억 7224만</t>
   </si>
   <si>
-    <t>고래털</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%B3%A0%EB%9E%98%ED%84%B8</t>
-  </si>
-  <si>
-    <t>295조 4654억 164만</t>
-  </si>
-  <si>
     <t>즐처드셈</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%EC%A6%90%EC%B2%98%EB%93%9C%EC%85%88</t>
   </si>
   <si>
-    <t>276조 4704억 5114만</t>
+    <t>277조 4730억 46만</t>
   </si>
   <si>
     <t>ADELL</t>
@@ -770,7 +770,16 @@
     <t>https://mgf.gg/contents/character.php?n=ADELL</t>
   </si>
   <si>
-    <t>256조 7707억</t>
+    <t>272조 2214억 1266만</t>
+  </si>
+  <si>
+    <t>원순철</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%9B%90%EC%88%9C%EC%B2%A0</t>
+  </si>
+  <si>
+    <t>225조 7419억 1797만</t>
   </si>
   <si>
     <t>술취한호랑이</t>
@@ -782,16 +791,7 @@
     <t>106</t>
   </si>
   <si>
-    <t>203조 329억 2295만</t>
-  </si>
-  <si>
-    <t>원순철</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%9B%90%EC%88%9C%EC%B2%A0</t>
-  </si>
-  <si>
-    <t>188조 7559억 5571만</t>
+    <t>217조 7725억 9984만</t>
   </si>
   <si>
     <t>유디티기찬</t>
@@ -854,7 +854,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%B0%95%EB%AF%B8%EC%AF%94</t>
   </si>
   <si>
-    <t>86조 4584억 7190만</t>
+    <t>87조 7548억 488만</t>
   </si>
   <si>
     <t>왓쳐</t>
@@ -872,7 +872,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%82%A4%EC%9A%B0%EB%8A%94%EA%B1%B4%EC%A7%88%EC%83%89</t>
   </si>
   <si>
-    <t>68조 5118억 839만</t>
+    <t>72조 2015억 1281만</t>
   </si>
   <si>
     <t>햄쓱이</t>
@@ -881,7 +881,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%96%84%EC%93%B1%EC%9D%B4</t>
   </si>
   <si>
-    <t>53조 3070억 6121만</t>
+    <t>54조 7086억 8334만</t>
   </si>
   <si>
     <t>수년</t>
@@ -890,7 +890,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%88%98%EB%85%84</t>
   </si>
   <si>
-    <t>34조 854억 2086만</t>
+    <t>37조 6097억 9325만</t>
   </si>
   <si>
     <t>쿠쏘야로로</t>
@@ -905,6 +905,276 @@
     <t>21조 4860억 2226만</t>
   </si>
   <si>
+    <t>가숭혁</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%B0%80%EC%88%AD%ED%98%81</t>
+  </si>
+  <si>
+    <t>5경 6927조 9409억 1785만</t>
+  </si>
+  <si>
+    <t>상탸치</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%83%81%ED%83%B8%EC%B9%98</t>
+  </si>
+  <si>
+    <t>1경 4800조 164억 9491만</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%82%B4%EB%BD%80%EC%8B%9C</t>
+  </si>
+  <si>
+    <t>1경 2977조 9849억 4944만</t>
+  </si>
+  <si>
+    <t>김우이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%B9%80%EC%9A%B0%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>8087조 1925억 4709만</t>
+  </si>
+  <si>
+    <t>26길초</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=26%EA%B8%B8%EC%B4%88</t>
+  </si>
+  <si>
+    <t>5398조 9067억 5787만</t>
+  </si>
+  <si>
+    <t>쑤린</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%91%A4%EB%A6%B0</t>
+  </si>
+  <si>
+    <t>4503조 8201억 8040만</t>
+  </si>
+  <si>
+    <t>뇌쉬</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%87%8C%EC%89%AC</t>
+  </si>
+  <si>
+    <t>3447조 8742억 5552만</t>
+  </si>
+  <si>
+    <t>한수찬</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%95%9C%EC%88%98%EC%B0%AC</t>
+  </si>
+  <si>
+    <t>2928조 3143억 4153만</t>
+  </si>
+  <si>
+    <t>중탸치</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A4%91%ED%83%B8%EC%B9%98</t>
+  </si>
+  <si>
+    <t>2746조 1096억 4932만</t>
+  </si>
+  <si>
+    <t>서예슬</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%84%9C%EC%98%88%EC%8A%AC</t>
+  </si>
+  <si>
+    <t>2298조 8130억 5066만</t>
+  </si>
+  <si>
+    <t>뻔수니</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%BB%94%EC%88%98%EB%8B%88</t>
+  </si>
+  <si>
+    <t>1619조 277억 6211만</t>
+  </si>
+  <si>
+    <t>라흐S2</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%9D%BC%ED%9D%90S2</t>
+  </si>
+  <si>
+    <t>1565조 1259억 3604만</t>
+  </si>
+  <si>
+    <t>한수린</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%95%9C%EC%88%98%EB%A6%B0</t>
+  </si>
+  <si>
+    <t>1439조 5237억 4055만</t>
+  </si>
+  <si>
+    <t>임승민</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%9E%84%EC%8A%B9%EB%AF%BC</t>
+  </si>
+  <si>
+    <t>1401조 9636억 9323만</t>
+  </si>
+  <si>
+    <t>덜박</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8D%9C%EB%B0%95</t>
+  </si>
+  <si>
+    <t>1225조 5378억 3431만</t>
+  </si>
+  <si>
+    <t>막탐</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A7%89%ED%83%90</t>
+  </si>
+  <si>
+    <t>보우마스터</t>
+  </si>
+  <si>
+    <t>605조 8844억 347만</t>
+  </si>
+  <si>
+    <t>쑤삔</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%91%A4%EC%82%94</t>
+  </si>
+  <si>
+    <t>314조 2935억 9965만</t>
+  </si>
+  <si>
+    <t>메키무라딘</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A9%94%ED%82%A4%EB%AC%B4%EB%9D%BC%EB%94%98</t>
+  </si>
+  <si>
+    <t>230조 4809억 9720만</t>
+  </si>
+  <si>
+    <t>륵스리</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A5%B5%EC%8A%A4%EB%A6%AC</t>
+  </si>
+  <si>
+    <t>219조 4232억 8026만</t>
+  </si>
+  <si>
+    <t>26배털</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=26%EB%B0%B0%ED%84%B8</t>
+  </si>
+  <si>
+    <t>218조 7034억 357만</t>
+  </si>
+  <si>
+    <t>류테</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A5%98%ED%85%8C</t>
+  </si>
+  <si>
+    <t>199조 7463억 9040만</t>
+  </si>
+  <si>
+    <t>26퐝바</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=26%ED%90%9D%EB%B0%94</t>
+  </si>
+  <si>
+    <t>198조 9629억 7530만</t>
+  </si>
+  <si>
+    <t>아모르파티퀘</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%95%84%EB%AA%A8%EB%A5%B4%ED%8C%8C%ED%8B%B0%ED%80%98</t>
+  </si>
+  <si>
+    <t>191조 4514억 5995만</t>
+  </si>
+  <si>
+    <t>뿜삐</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%BF%9C%EC%82%90</t>
+  </si>
+  <si>
+    <t>166조 9906억 8312만</t>
+  </si>
+  <si>
+    <t>최씨용</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%B5%9C%EC%94%A8%EC%9A%A9</t>
+  </si>
+  <si>
+    <t>165조 3399억 4755만</t>
+  </si>
+  <si>
+    <t>뻐늬</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%BB%90%EB%8A%AC</t>
+  </si>
+  <si>
+    <t>161조 401억 2061만</t>
+  </si>
+  <si>
+    <t>브깃</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%B8%8C%EA%B9%83</t>
+  </si>
+  <si>
+    <t>97조 7245억 6292만</t>
+  </si>
+  <si>
+    <t>반석동회주먹</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%B0%98%EC%84%9D%EB%8F%99%ED%9A%8C%EC%A3%BC%EB%A8%B9</t>
+  </si>
+  <si>
+    <t>62조 4045억 7236만</t>
+  </si>
+  <si>
+    <t>서이따</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%84%9C%EC%9D%B4%EB%94%B0</t>
+  </si>
+  <si>
+    <t>50조 3859억 842만</t>
+  </si>
+  <si>
+    <t>예라미</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%98%88%EB%9D%BC%EB%AF%B8</t>
+  </si>
+  <si>
+    <t>50조 499억 6960만</t>
+  </si>
+  <si>
     <t>https://mgf.gg/contents/character.php?n=%EB%AC%B4%EC%B9%98z</t>
   </si>
   <si>
@@ -917,7 +1187,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%9E%84%EC%88%9C%EC%9D%B4</t>
   </si>
   <si>
-    <t>9418조 7414억 1411만</t>
+    <t>9839조 8942억 771만</t>
   </si>
   <si>
     <t>쥬정뱅이</t>
@@ -935,7 +1205,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EA%B7%80%EC%97%AC%EC%9B%8C%EC%84%9C%EB%AF%B8%EC%95%88</t>
   </si>
   <si>
-    <t>6795조 6367억 9500만</t>
+    <t>6831조 2701억 6272만</t>
   </si>
   <si>
     <t>밀프푸씨</t>
@@ -944,7 +1214,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%B0%80%ED%94%84%ED%91%B8%EC%94%A8</t>
   </si>
   <si>
-    <t>3993조 434억 9397만</t>
+    <t>4207조 3406억 646만</t>
   </si>
   <si>
     <t>쑥국</t>
@@ -989,7 +1259,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%9D%BC%EC%84%B8%EB%8A%90</t>
   </si>
   <si>
-    <t>1278조 3516억 5059만</t>
+    <t>1279조 566억 7216만</t>
   </si>
   <si>
     <t>엔젤가든</t>
@@ -998,7 +1268,16 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%97%94%EC%A0%A4%EA%B0%80%EB%93%A0</t>
   </si>
   <si>
-    <t>1173조 7781억 9023만</t>
+    <t>1178조 1172억 6506만</t>
+  </si>
+  <si>
+    <t>핫장</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%95%AB%EC%9E%A5</t>
+  </si>
+  <si>
+    <t>1060조 8243억 8674만</t>
   </si>
   <si>
     <t>약해진쭌석</t>
@@ -1010,6 +1289,15 @@
     <t>1058조 9827억 7836만</t>
   </si>
   <si>
+    <t>냉도</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%83%89%EB%8F%84</t>
+  </si>
+  <si>
+    <t>1058조 1099억 1237만</t>
+  </si>
+  <si>
     <t>노득</t>
   </si>
   <si>
@@ -1019,22 +1307,13 @@
     <t>1046조 8188억 6403만</t>
   </si>
   <si>
-    <t>냉도</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%83%89%EB%8F%84</t>
-  </si>
-  <si>
-    <t>1036조 8523억 1530만</t>
-  </si>
-  <si>
-    <t>핫장</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%95%AB%EC%9E%A5</t>
-  </si>
-  <si>
-    <t>990조 4775억 3465만</t>
+    <t>사진쟁이</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%82%AC%EC%A7%84%EC%9F%81%EC%9D%B4</t>
+  </si>
+  <si>
+    <t>994조 8405억 3318만</t>
   </si>
   <si>
     <t>피치에이드</t>
@@ -1043,16 +1322,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%94%BC%EC%B9%98%EC%97%90%EC%9D%B4%EB%93%9C</t>
   </si>
   <si>
-    <t>966조 3304억 9738만</t>
-  </si>
-  <si>
-    <t>사진쟁이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%82%AC%EC%A7%84%EC%9F%81%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>894조 4251억 2035만</t>
+    <t>968조 7142억 2266만</t>
   </si>
   <si>
     <t>겸찰</t>
@@ -1079,7 +1349,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%97%9B%EC%A0%90</t>
   </si>
   <si>
-    <t>697조 7467억 5290만</t>
+    <t>698조 3664억 7232만</t>
   </si>
   <si>
     <t>키은</t>
@@ -1106,7 +1376,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EA%B0%9C%EC%A0%90</t>
   </si>
   <si>
-    <t>462조 5936억 1315만</t>
+    <t>469조 8226억 287만</t>
   </si>
   <si>
     <t>챠재범</t>
@@ -1115,7 +1385,16 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%B1%A0%EC%9E%AC%EB%B2%94</t>
   </si>
   <si>
-    <t>414조 4879억 5258만</t>
+    <t>417조 8498억 1125만</t>
+  </si>
+  <si>
+    <t>사마련</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%82%AC%EB%A7%88%EB%A0%A8</t>
+  </si>
+  <si>
+    <t>394조 5420억 8183만</t>
   </si>
   <si>
     <t>81학찬</t>
@@ -1127,22 +1406,13 @@
     <t>384조 7178억 1530만</t>
   </si>
   <si>
-    <t>사마련</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%82%AC%EB%A7%88%EB%A0%A8</t>
-  </si>
-  <si>
-    <t>356조 1208억 1892만</t>
-  </si>
-  <si>
     <t>머쓰윽타드</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%EB%A8%B8%EC%93%B0%EC%9C%BD%ED%83%80%EB%93%9C</t>
   </si>
   <si>
-    <t>336조 8694억 6083만</t>
+    <t>375조 7409억 1664만</t>
   </si>
   <si>
     <t>쵸꼬님</t>
@@ -1172,276 +1442,6 @@
     <t>135조 3248억 3228만</t>
   </si>
   <si>
-    <t>가숭혁</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%B0%80%EC%88%AD%ED%98%81</t>
-  </si>
-  <si>
-    <t>5경 6927조 9409억 1785만</t>
-  </si>
-  <si>
-    <t>상탸치</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%83%81%ED%83%B8%EC%B9%98</t>
-  </si>
-  <si>
-    <t>1경 4800조 164억 9491만</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%82%B4%EB%BD%80%EC%8B%9C</t>
-  </si>
-  <si>
-    <t>1경 2977조 9849억 4944만</t>
-  </si>
-  <si>
-    <t>김우이</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%B9%80%EC%9A%B0%EC%9D%B4</t>
-  </si>
-  <si>
-    <t>7846조 3950억 9885만</t>
-  </si>
-  <si>
-    <t>26길초</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=26%EA%B8%B8%EC%B4%88</t>
-  </si>
-  <si>
-    <t>5172조 5777억 827만</t>
-  </si>
-  <si>
-    <t>쑤린</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%91%A4%EB%A6%B0</t>
-  </si>
-  <si>
-    <t>4503조 8201억 8040만</t>
-  </si>
-  <si>
-    <t>뇌쉬</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%87%8C%EC%89%AC</t>
-  </si>
-  <si>
-    <t>3447조 8742억 5552만</t>
-  </si>
-  <si>
-    <t>한수찬</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%95%9C%EC%88%98%EC%B0%AC</t>
-  </si>
-  <si>
-    <t>2879조 8534억 3444만</t>
-  </si>
-  <si>
-    <t>중탸치</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A4%91%ED%83%B8%EC%B9%98</t>
-  </si>
-  <si>
-    <t>2744조 4086억 7914만</t>
-  </si>
-  <si>
-    <t>서예슬</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%84%9C%EC%98%88%EC%8A%AC</t>
-  </si>
-  <si>
-    <t>2293조 2557억 7607만</t>
-  </si>
-  <si>
-    <t>한수린</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%95%9C%EC%88%98%EB%A6%B0</t>
-  </si>
-  <si>
-    <t>1431조 5415억 918만</t>
-  </si>
-  <si>
-    <t>뻔수니</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%BB%94%EC%88%98%EB%8B%88</t>
-  </si>
-  <si>
-    <t>1402조 5178억 1235만</t>
-  </si>
-  <si>
-    <t>임승민</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%9E%84%EC%8A%B9%EB%AF%BC</t>
-  </si>
-  <si>
-    <t>1401조 9636억 9323만</t>
-  </si>
-  <si>
-    <t>덜박</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8D%9C%EB%B0%95</t>
-  </si>
-  <si>
-    <t>1186조 1413억 1739만</t>
-  </si>
-  <si>
-    <t>라흐S2</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%9D%BC%ED%9D%90S2</t>
-  </si>
-  <si>
-    <t>1121조 5538억 750만</t>
-  </si>
-  <si>
-    <t>막탐</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A7%89%ED%83%90</t>
-  </si>
-  <si>
-    <t>보우마스터</t>
-  </si>
-  <si>
-    <t>605조 8844억 347만</t>
-  </si>
-  <si>
-    <t>쑤삔</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%91%A4%EC%82%94</t>
-  </si>
-  <si>
-    <t>314조 2935억 9965만</t>
-  </si>
-  <si>
-    <t>메키무라딘</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A9%94%ED%82%A4%EB%AC%B4%EB%9D%BC%EB%94%98</t>
-  </si>
-  <si>
-    <t>230조 4809억 9720만</t>
-  </si>
-  <si>
-    <t>륵스리</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A5%B5%EC%8A%A4%EB%A6%AC</t>
-  </si>
-  <si>
-    <t>219조 4232억 8026만</t>
-  </si>
-  <si>
-    <t>26배털</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=26%EB%B0%B0%ED%84%B8</t>
-  </si>
-  <si>
-    <t>218조 7034억 357만</t>
-  </si>
-  <si>
-    <t>류테</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A5%98%ED%85%8C</t>
-  </si>
-  <si>
-    <t>199조 152억 4793만</t>
-  </si>
-  <si>
-    <t>26퐝바</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=26%ED%90%9D%EB%B0%94</t>
-  </si>
-  <si>
-    <t>198조 9629억 7530만</t>
-  </si>
-  <si>
-    <t>아모르파티퀘</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%95%84%EB%AA%A8%EB%A5%B4%ED%8C%8C%ED%8B%B0%ED%80%98</t>
-  </si>
-  <si>
-    <t>191조 4514억 5995만</t>
-  </si>
-  <si>
-    <t>뿜삐</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%BF%9C%EC%82%90</t>
-  </si>
-  <si>
-    <t>163조 5507억 1900만</t>
-  </si>
-  <si>
-    <t>최씨용</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%B5%9C%EC%94%A8%EC%9A%A9</t>
-  </si>
-  <si>
-    <t>162조 8305억 2169만</t>
-  </si>
-  <si>
-    <t>뻐늬</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%BB%90%EB%8A%AC</t>
-  </si>
-  <si>
-    <t>160조 8583억 7003만</t>
-  </si>
-  <si>
-    <t>브깃</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%B8%8C%EA%B9%83</t>
-  </si>
-  <si>
-    <t>97조 7245억 6292만</t>
-  </si>
-  <si>
-    <t>반석동회주먹</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%B0%98%EC%84%9D%EB%8F%99%ED%9A%8C%EC%A3%BC%EB%A8%B9</t>
-  </si>
-  <si>
-    <t>60조 3230억 3149만</t>
-  </si>
-  <si>
-    <t>서이따</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%84%9C%EC%9D%B4%EB%94%B0</t>
-  </si>
-  <si>
-    <t>50조 3859억 842만</t>
-  </si>
-  <si>
-    <t>예라미</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%98%88%EB%9D%BC%EB%AF%B8</t>
-  </si>
-  <si>
-    <t>44조 9829억 3334만</t>
-  </si>
-  <si>
     <t>주의력</t>
   </si>
   <si>
@@ -1457,7 +1457,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%8A%A8%EB%85%80</t>
   </si>
   <si>
-    <t>2경 5688조 6031억 4759만</t>
+    <t>2경 6471조 3334억 2068만</t>
   </si>
   <si>
     <t>맠스맨</t>
@@ -1502,7 +1502,16 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%8F%84%EB%A0%B93</t>
   </si>
   <si>
-    <t>366조 2039억 2073만</t>
+    <t>448조 4296억 8084만</t>
+  </si>
+  <si>
+    <t>엘리자베타</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%97%98%EB%A6%AC%EC%9E%90%EB%B2%A0%ED%83%80</t>
+  </si>
+  <si>
+    <t>423조 5685억 1379만</t>
   </si>
   <si>
     <t>천두</t>
@@ -1511,16 +1520,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%B2%9C%EB%91%90</t>
   </si>
   <si>
-    <t>357조 3804억 8258만</t>
-  </si>
-  <si>
-    <t>엘리자베타</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%97%98%EB%A6%AC%EC%9E%90%EB%B2%A0%ED%83%80</t>
-  </si>
-  <si>
-    <t>341조 9233억 3947만</t>
+    <t>421조 8869억 713만</t>
   </si>
   <si>
     <t>o엔젤o</t>
@@ -1529,7 +1529,7 @@
     <t>https://mgf.gg/contents/character.php?n=o%EC%97%94%EC%A0%A4o</t>
   </si>
   <si>
-    <t>319조 9744억 9530만</t>
+    <t>371조 3013억 3443만</t>
   </si>
   <si>
     <t>이러는거아냐</t>
@@ -1556,7 +1556,7 @@
     <t>https://mgf.gg/contents/character.php?n=24%EB%85%84%EC%83%9D%EC%A0%95%EC%B6%98%EC%8B%9D</t>
   </si>
   <si>
-    <t>244조 7515억 7699만</t>
+    <t>251조 1978억 6824만</t>
   </si>
   <si>
     <t>키움맨</t>
@@ -1568,22 +1568,22 @@
     <t>221조 4644억 9402만</t>
   </si>
   <si>
+    <t>한유화</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%ED%95%9C%EC%9C%A0%ED%99%94</t>
+  </si>
+  <si>
+    <t>130조 8703억 8412만</t>
+  </si>
+  <si>
     <t>혈마신</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%ED%98%88%EB%A7%88%EC%8B%A0</t>
   </si>
   <si>
-    <t>123조 6016억 7284만</t>
-  </si>
-  <si>
-    <t>한유화</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%ED%95%9C%EC%9C%A0%ED%99%94</t>
-  </si>
-  <si>
-    <t>121조 3528억 4933만</t>
+    <t>125조 7012억 5379만</t>
   </si>
   <si>
     <t>숮2</t>
@@ -1598,28 +1598,37 @@
     <t>116조 1641억 4298만</t>
   </si>
   <si>
+    <t>리얼크크</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%A6%AC%EC%96%BC%ED%81%AC%ED%81%AC</t>
+  </si>
+  <si>
+    <t>102조 8690억 1004만</t>
+  </si>
+  <si>
     <t>현즈</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%ED%98%84%EC%A6%88</t>
   </si>
   <si>
-    <t>101조 2265억 9420만</t>
-  </si>
-  <si>
-    <t>리얼크크</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%A6%AC%EC%96%BC%ED%81%AC%ED%81%AC</t>
-  </si>
-  <si>
-    <t>92조 140억 8811만</t>
+    <t>101조 4445억 4537만</t>
+  </si>
+  <si>
+    <t>쩔뚝</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EC%A9%94%EB%9A%9D</t>
+  </si>
+  <si>
+    <t>89조 8851억 2967만</t>
   </si>
   <si>
     <t>https://mgf.gg/contents/character.php?n=%ED%86%A0%EB%A7%88%EC%8A%A4%EC%85%B8%EB%B9%84</t>
   </si>
   <si>
-    <t>76조 2071억 1665만</t>
+    <t>79조 4979억 5198만</t>
   </si>
   <si>
     <t>김똔똔</t>
@@ -1628,28 +1637,19 @@
     <t>https://mgf.gg/contents/character.php?n=%EA%B9%80%EB%98%94%EB%98%94</t>
   </si>
   <si>
-    <t>65조 8628억 2420만</t>
-  </si>
-  <si>
-    <t>쩔뚝</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EC%A9%94%EB%9A%9D</t>
+    <t>69조 7229억 6939만</t>
+  </si>
+  <si>
+    <t>니코짱</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%8B%88%EC%BD%94%EC%A7%B1</t>
   </si>
   <si>
     <t>104</t>
   </si>
   <si>
-    <t>64조 9381억 8304만</t>
-  </si>
-  <si>
-    <t>니코짱</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%8B%88%EC%BD%94%EC%A7%B1</t>
-  </si>
-  <si>
-    <t>49조 1483억 9285만</t>
+    <t>49조 6787억 1436만</t>
   </si>
   <si>
     <t>박하민린</t>
@@ -1667,7 +1667,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%B9%B4%EA%B5%AC%EC%96%91</t>
   </si>
   <si>
-    <t>37조 5638억 4062만</t>
+    <t>40조 5712억 1159만</t>
   </si>
   <si>
     <t>Vv번걔의신vV</t>
@@ -1676,7 +1676,7 @@
     <t>https://mgf.gg/contents/character.php?n=Vv%EB%B2%88%EA%B1%94%EC%9D%98%EC%8B%A0vV</t>
   </si>
   <si>
-    <t>37조 2957억 8253만</t>
+    <t>39조 1718억 9172만</t>
   </si>
   <si>
     <t>오빠내꼬</t>
@@ -1703,7 +1703,7 @@
     <t>https://mgf.gg/contents/character.php?n=%ED%97%88%EC%9C%B0</t>
   </si>
   <si>
-    <t>18조 2939억 9789만</t>
+    <t>18조 3247억 1002만</t>
   </si>
   <si>
     <t>뉴맹우</t>
@@ -2234,22 +2234,22 @@
         <v>36</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>24</v>
@@ -2257,28 +2257,28 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>20</v>
@@ -2644,10 +2644,10 @@
         <v>73</v>
       </c>
       <c r="H9" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>24</v>
@@ -2658,16 +2658,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>66</v>
@@ -2676,7 +2676,7 @@
         <v>89</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>109</v>
@@ -2804,7 +2804,7 @@
         <v>89</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>128</v>
@@ -2836,7 +2836,7 @@
         <v>79</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>132</v>
@@ -2932,7 +2932,7 @@
         <v>89</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>145</v>
@@ -3028,7 +3028,7 @@
         <v>73</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>149</v>
+        <v>114</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>158</v>
@@ -3074,16 +3074,16 @@
         <v>13</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>66</v>
@@ -3095,7 +3095,7 @@
         <v>149</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>24</v>
@@ -3106,7 +3106,7 @@
         <v>13</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>17</v>
+        <v>165</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>166</v>
@@ -3202,7 +3202,7 @@
         <v>13</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>23</v>
@@ -3220,10 +3220,10 @@
         <v>73</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>24</v>
@@ -3234,16 +3234,16 @@
         <v>13</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>66</v>
@@ -3252,10 +3252,10 @@
         <v>140</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>24</v>
@@ -3266,16 +3266,16 @@
         <v>13</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>66</v>
@@ -3284,7 +3284,7 @@
         <v>89</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>189</v>
@@ -3348,7 +3348,7 @@
         <v>73</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>198</v>
@@ -3406,7 +3406,7 @@
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="50.7109375" customWidth="1"/>
     <col min="6" max="8" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3657,7 +3657,7 @@
         <v>79</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>220</v>
@@ -3703,7 +3703,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>224</v>
@@ -3721,7 +3721,7 @@
         <v>89</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>226</v>
@@ -3753,7 +3753,7 @@
         <v>67</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>229</v>
@@ -3785,7 +3785,7 @@
         <v>73</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>232</v>
@@ -3846,10 +3846,10 @@
         <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>79</v>
+        <v>140</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>238</v>
@@ -3878,7 +3878,7 @@
         <v>66</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>140</v>
+        <v>79</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>168</v>
@@ -3913,7 +3913,7 @@
         <v>73</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>244</v>
@@ -3945,7 +3945,7 @@
         <v>119</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>247</v>
@@ -3977,10 +3977,10 @@
         <v>89</v>
       </c>
       <c r="H18" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>24</v>
@@ -3994,13 +3994,13 @@
         <v>146</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>253</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>66</v>
@@ -4009,7 +4009,7 @@
         <v>89</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>168</v>
+        <v>253</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>254</v>
@@ -4041,7 +4041,7 @@
         <v>79</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>257</v>
@@ -4073,7 +4073,7 @@
         <v>67</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>260</v>
@@ -4119,7 +4119,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>162</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>264</v>
@@ -4137,7 +4137,7 @@
         <v>119</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>266</v>
@@ -4151,7 +4151,7 @@
         <v>25</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>17</v>
+        <v>165</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>267</v>
@@ -4169,7 +4169,7 @@
         <v>119</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>269</v>
@@ -4233,7 +4233,7 @@
         <v>140</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>275</v>
@@ -4247,7 +4247,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>276</v>
@@ -4265,7 +4265,7 @@
         <v>89</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>278</v>
@@ -4279,7 +4279,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>279</v>
@@ -4297,7 +4297,7 @@
         <v>140</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>281</v>
@@ -4311,7 +4311,7 @@
         <v>25</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>282</v>
@@ -4361,7 +4361,7 @@
         <v>140</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>287</v>
@@ -4451,7 +4451,7 @@
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="50.7109375" customWidth="1"/>
     <col min="6" max="8" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4495,25 +4495,25 @@
         <v>63</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>40</v>
+        <v>292</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>40</v>
+        <v>292</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>179</v>
+        <v>66</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>68</v>
+        <v>200</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>24</v>
@@ -4527,25 +4527,25 @@
         <v>70</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>24</v>
@@ -4559,22 +4559,22 @@
         <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>297</v>
+        <v>39</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>297</v>
+        <v>39</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>298</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>66</v>
+        <v>179</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>299</v>
@@ -4603,10 +4603,10 @@
         <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>90</v>
+        <v>216</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>302</v>
@@ -4635,7 +4635,7 @@
         <v>66</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>95</v>
@@ -4667,10 +4667,10 @@
         <v>66</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>308</v>
@@ -4699,10 +4699,10 @@
         <v>66</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>216</v>
+        <v>95</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>311</v>
@@ -4734,7 +4734,7 @@
         <v>73</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>314</v>
@@ -4748,7 +4748,7 @@
         <v>33</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>315</v>
@@ -4766,7 +4766,7 @@
         <v>73</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>317</v>
@@ -4798,7 +4798,7 @@
         <v>73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>320</v>
@@ -4830,7 +4830,7 @@
         <v>89</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>323</v>
@@ -4862,7 +4862,7 @@
         <v>73</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>326</v>
@@ -4891,10 +4891,10 @@
         <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>149</v>
+        <v>108</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>329</v>
@@ -4926,7 +4926,7 @@
         <v>89</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>332</v>
@@ -4955,10 +4955,10 @@
         <v>66</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>335</v>
@@ -4987,13 +4987,13 @@
         <v>66</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>67</v>
+        <v>338</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>114</v>
+        <v>180</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>24</v>
@@ -5007,25 +5007,25 @@
         <v>142</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>114</v>
+        <v>168</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>24</v>
@@ -5039,25 +5039,25 @@
         <v>146</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>114</v>
+        <v>180</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>24</v>
@@ -5071,25 +5071,25 @@
         <v>151</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>24</v>
@@ -5103,25 +5103,25 @@
         <v>155</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>24</v>
@@ -5135,25 +5135,25 @@
         <v>28</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>114</v>
+        <v>168</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>24</v>
@@ -5164,16 +5164,16 @@
         <v>33</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>162</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>66</v>
@@ -5182,10 +5182,10 @@
         <v>73</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>114</v>
+        <v>168</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>24</v>
@@ -5196,28 +5196,28 @@
         <v>33</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>17</v>
+        <v>165</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>114</v>
+        <v>168</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>24</v>
@@ -5231,25 +5231,25 @@
         <v>170</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>24</v>
@@ -5263,25 +5263,25 @@
         <v>51</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>24</v>
@@ -5292,28 +5292,28 @@
         <v>33</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>24</v>
@@ -5324,28 +5324,28 @@
         <v>33</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>73</v>
+        <v>338</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>149</v>
+        <v>253</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>24</v>
@@ -5356,28 +5356,28 @@
         <v>33</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>24</v>
@@ -5391,25 +5391,25 @@
         <v>190</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>24</v>
@@ -5423,25 +5423,25 @@
         <v>195</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>188</v>
+        <v>253</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>24</v>
@@ -5496,7 +5496,7 @@
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="50.7109375" customWidth="1"/>
     <col min="6" max="8" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5534,28 +5534,28 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>381</v>
+        <v>47</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>381</v>
+        <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>382</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>66</v>
+        <v>179</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>383</v>
@@ -5566,7 +5566,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>70</v>
@@ -5584,10 +5584,10 @@
         <v>66</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>386</v>
@@ -5598,31 +5598,31 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>47</v>
+        <v>387</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>47</v>
+        <v>387</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>179</v>
+        <v>66</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>24</v>
@@ -5630,31 +5630,31 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>82</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>216</v>
+        <v>90</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>24</v>
@@ -5662,31 +5662,31 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>95</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>24</v>
@@ -5694,31 +5694,31 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>92</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>24</v>
@@ -5726,31 +5726,31 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>97</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>95</v>
+        <v>216</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>24</v>
@@ -5758,19 +5758,19 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>66</v>
@@ -5779,10 +5779,10 @@
         <v>73</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>24</v>
@@ -5790,19 +5790,19 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>66</v>
@@ -5811,10 +5811,10 @@
         <v>73</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>24</v>
@@ -5822,19 +5822,19 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>66</v>
@@ -5843,10 +5843,10 @@
         <v>73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>24</v>
@@ -5854,31 +5854,31 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>116</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>24</v>
@@ -5886,31 +5886,31 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>114</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>24</v>
@@ -5918,31 +5918,31 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>24</v>
@@ -5950,31 +5950,31 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>129</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>24</v>
@@ -5982,31 +5982,31 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>133</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>188</v>
+        <v>149</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>24</v>
@@ -6014,28 +6014,28 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>66</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>427</v>
+        <v>79</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>168</v>
+        <v>114</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>428</v>
@@ -6046,7 +6046,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>142</v>
@@ -6064,10 +6064,10 @@
         <v>66</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>188</v>
+        <v>114</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>431</v>
@@ -6078,7 +6078,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>146</v>
@@ -6096,10 +6096,10 @@
         <v>66</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>168</v>
+        <v>114</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>434</v>
@@ -6110,7 +6110,7 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>151</v>
@@ -6128,10 +6128,10 @@
         <v>66</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>149</v>
+        <v>114</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>437</v>
@@ -6142,7 +6142,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>155</v>
@@ -6160,10 +6160,10 @@
         <v>66</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>149</v>
+        <v>114</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>440</v>
@@ -6174,7 +6174,7 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>28</v>
@@ -6192,10 +6192,10 @@
         <v>66</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>188</v>
+        <v>114</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>443</v>
@@ -6206,10 +6206,10 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>162</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>444</v>
@@ -6227,7 +6227,7 @@
         <v>73</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>188</v>
+        <v>114</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>446</v>
@@ -6238,10 +6238,10 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>17</v>
+        <v>165</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>447</v>
@@ -6256,10 +6256,10 @@
         <v>66</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>188</v>
+        <v>114</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>449</v>
@@ -6270,7 +6270,7 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>170</v>
@@ -6288,7 +6288,7 @@
         <v>66</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>168</v>
@@ -6302,7 +6302,7 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>51</v>
@@ -6320,10 +6320,10 @@
         <v>66</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>455</v>
@@ -6334,10 +6334,10 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>456</v>
@@ -6352,10 +6352,10 @@
         <v>66</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>89</v>
+        <v>140</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>458</v>
@@ -6366,10 +6366,10 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>459</v>
@@ -6384,10 +6384,10 @@
         <v>66</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>427</v>
+        <v>73</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>250</v>
+        <v>149</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>461</v>
@@ -6398,10 +6398,10 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>462</v>
@@ -6416,10 +6416,10 @@
         <v>66</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>464</v>
@@ -6430,7 +6430,7 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>190</v>
@@ -6448,10 +6448,10 @@
         <v>66</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>467</v>
@@ -6462,7 +6462,7 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>195</v>
@@ -6480,10 +6480,10 @@
         <v>66</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>140</v>
+        <v>67</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>470</v>
@@ -6693,10 +6693,10 @@
         <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>482</v>
@@ -6760,7 +6760,7 @@
         <v>73</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>488</v>
@@ -6821,10 +6821,10 @@
         <v>66</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>188</v>
+        <v>149</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>494</v>
@@ -6838,7 +6838,7 @@
         <v>48</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>495</v>
@@ -6853,10 +6853,10 @@
         <v>66</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>497</v>
@@ -6888,7 +6888,7 @@
         <v>73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>500</v>
@@ -6920,7 +6920,7 @@
         <v>119</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>503</v>
@@ -6952,7 +6952,7 @@
         <v>119</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>506</v>
@@ -6984,7 +6984,7 @@
         <v>73</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>509</v>
@@ -7016,7 +7016,7 @@
         <v>89</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>512</v>
@@ -7045,10 +7045,10 @@
         <v>66</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>73</v>
+        <v>140</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>168</v>
+        <v>253</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>515</v>
@@ -7077,10 +7077,10 @@
         <v>66</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>250</v>
+        <v>168</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>518</v>
@@ -7112,7 +7112,7 @@
         <v>521</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>522</v>
@@ -7141,10 +7141,10 @@
         <v>66</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>525</v>
@@ -7173,10 +7173,10 @@
         <v>66</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>528</v>
@@ -7193,25 +7193,25 @@
         <v>155</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>54</v>
+        <v>529</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>54</v>
+        <v>529</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>179</v>
+        <v>66</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>24</v>
@@ -7225,22 +7225,22 @@
         <v>28</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>531</v>
+        <v>54</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>531</v>
+        <v>54</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>532</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>66</v>
+        <v>179</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>533</v>
@@ -7254,7 +7254,7 @@
         <v>48</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>162</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>534</v>
@@ -7269,13 +7269,13 @@
         <v>66</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H23" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>536</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>537</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>24</v>
@@ -7286,16 +7286,16 @@
         <v>48</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>17</v>
+        <v>165</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>538</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>539</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>66</v>
@@ -7304,7 +7304,7 @@
         <v>140</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>540</v>
@@ -7368,7 +7368,7 @@
         <v>89</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>546</v>
@@ -7382,7 +7382,7 @@
         <v>48</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>547</v>
@@ -7397,10 +7397,10 @@
         <v>66</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>427</v>
+        <v>338</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>549</v>
@@ -7414,7 +7414,7 @@
         <v>48</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>550</v>
@@ -7446,7 +7446,7 @@
         <v>48</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>553</v>
@@ -7464,7 +7464,7 @@
         <v>119</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>555</v>

</xml_diff>